<commit_message>
Add coverage gate to CI
</commit_message>
<xml_diff>
--- a/data/sample_inventory.xlsx
+++ b/data/sample_inventory.xlsx
@@ -542,20 +542,20 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>2026-06-03 22:49:42</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n">
         <v>41</v>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>2026-06-03 22:40:29</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>Alex</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>44</v>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
@@ -736,16 +736,16 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>2026-06-03 22:40:29</t>
+          <t>2026-06-03 22:49:42</t>
         </is>
       </c>
       <c r="E11" s="1" t="n"/>
       <c r="F11" s="1" t="n">
-        <v>326</v>
+        <v>336</v>
       </c>
       <c r="G11" s="1" t="n"/>
     </row>
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1006,36 +1006,40 @@
       <c r="G6" s="4" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:10:57</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>S023</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Strawberry</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-03 22:49:42</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Cherry</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03 15:42:45</t>
+          <t>2026-06-03 00:10:57</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1062,7 +1066,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03 15:43:52</t>
+          <t>2026-06-03 15:42:45</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -1089,7 +1093,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03 22:40:05</t>
+          <t>2026-06-03 15:43:52</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1116,7 +1120,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03 22:40:29</t>
+          <t>2026-06-03 22:40:05</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1139,6 +1143,60 @@
       </c>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03 22:40:29</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Strawberry</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03 22:49:42</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Strawberry</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: update README and clarify manual DB checks
</commit_message>
<xml_diff>
--- a/data/sample_inventory.xlsx
+++ b/data/sample_inventory.xlsx
@@ -542,11 +542,11 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>2026-06-03 22:49:42</t>
+          <t>2026-06-09 23:24:41</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr">
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="F3" s="1" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
@@ -736,16 +736,16 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>346</v>
+        <v>366</v>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>2026-06-03 22:49:42</t>
+          <t>2026-06-09 23:24:41</t>
         </is>
       </c>
       <c r="E11" s="1" t="n"/>
       <c r="F11" s="1" t="n">
-        <v>336</v>
+        <v>356</v>
       </c>
       <c r="G11" s="1" t="n"/>
     </row>
@@ -806,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1037,63 +1037,71 @@
       <c r="G7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-03 00:10:57</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>S023</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Strawberry</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 23:14:26</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Cherry</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-03 15:42:45</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>S023</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Strawberry</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-09 23:24:41</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>C001</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Cherry</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03 15:43:52</t>
+          <t>2026-06-03 00:10:57</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1120,7 +1128,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03 22:40:05</t>
+          <t>2026-06-03 15:42:45</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -1147,7 +1155,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03 22:40:29</t>
+          <t>2026-06-03 15:43:52</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1174,7 +1182,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-03 22:49:42</t>
+          <t>2026-06-03 22:40:05</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1197,6 +1205,114 @@
       </c>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03 22:40:29</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Strawberry</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-03 22:49:42</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Strawberry</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09 23:14:26</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Strawberry</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-09 23:24:41</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>S023</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Strawberry</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>